<commit_message>
auto: Claude 코드 수정
</commit_message>
<xml_diff>
--- a/군사영어_전체데이터_20260511 (1,2주차 일부 포함).xlsx
+++ b/군사영어_전체데이터_20260511 (1,2주차 일부 포함).xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:C4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -409,13 +409,19 @@
       <c r="B1" t="str">
         <v>실행 일시</v>
       </c>
+      <c r="C1" t="str">
+        <v>_실행일시</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
         <v>1회차(6주차)</v>
       </c>
       <c r="B2" t="str">
-        <v>26. 04. 08. 오후 09:25</v>
+        <v>26. 04. 09. 오후 07:00</v>
+      </c>
+      <c r="C2" t="str">
+        <v>2026-04-09T19:00:00</v>
       </c>
     </row>
     <row r="3">
@@ -425,25 +431,31 @@
       <c r="B3" t="str">
         <v>26. 04. 16. 오후 07:00</v>
       </c>
+      <c r="C3" t="str">
+        <v>2026-04-16T19:00:00</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
         <v>3회차(10주차)</v>
       </c>
       <c r="B4" t="str">
-        <v>26. 05. 07. 오후 06:32</v>
+        <v>26. 05. 07. 오후 07:00</v>
+      </c>
+      <c r="C4" t="str">
+        <v>2026-05-07T19:00:00</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C4"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:F17"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -461,27 +473,33 @@
       <c r="E1" t="str">
         <v>당첨 일시</v>
       </c>
+      <c r="F1" t="str">
+        <v>_당첨일시</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
         <v>1회차(6주차)</v>
       </c>
       <c r="B2" t="str">
-        <v>24312005</v>
+        <v>24312004</v>
       </c>
       <c r="C2" t="str">
-        <v>김수빈</v>
+        <v>김석주</v>
       </c>
       <c r="D2" t="str">
-        <v>null번</v>
+        <v>-</v>
       </c>
       <c r="E2" t="str">
-        <v>26. 04. 08. 오후 09:25</v>
+        <v>26. 04. 09. 오후 07:00</v>
+      </c>
+      <c r="F2" t="str">
+        <v>2026-04-09T19:00:00</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>2회차(7주차)</v>
+        <v>1회차(6주차)</v>
       </c>
       <c r="B3" t="str">
         <v>24312005</v>
@@ -490,129 +508,153 @@
         <v>김수빈</v>
       </c>
       <c r="D3" t="str">
-        <v>null번</v>
+        <v>-</v>
       </c>
       <c r="E3" t="str">
-        <v>26. 04. 16. 오후 07:00</v>
+        <v>26. 04. 09. 오후 07:00</v>
+      </c>
+      <c r="F3" t="str">
+        <v>2026-04-09T19:00:00</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>2회차(7주차)</v>
+        <v>1회차(6주차)</v>
       </c>
       <c r="B4" t="str">
-        <v>24312006</v>
+        <v>24312009</v>
       </c>
       <c r="C4" t="str">
-        <v>김유정</v>
+        <v>남진서</v>
       </c>
       <c r="D4" t="str">
-        <v>null번</v>
+        <v>-</v>
       </c>
       <c r="E4" t="str">
-        <v>26. 04. 16. 오후 07:00</v>
+        <v>26. 04. 09. 오후 07:00</v>
+      </c>
+      <c r="F4" t="str">
+        <v>2026-04-09T19:00:00</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>2회차(7주차)</v>
+        <v>1회차(6주차)</v>
       </c>
       <c r="B5" t="str">
-        <v>24312022</v>
+        <v>24312010</v>
       </c>
       <c r="C5" t="str">
-        <v>변여아</v>
+        <v>박지민</v>
       </c>
       <c r="D5" t="str">
-        <v>null번</v>
+        <v>-</v>
       </c>
       <c r="E5" t="str">
-        <v>26. 04. 16. 오후 07:00</v>
+        <v>26. 04. 09. 오후 07:00</v>
+      </c>
+      <c r="F5" t="str">
+        <v>2026-04-09T19:00:00</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>3회차(10주차)</v>
+        <v>2회차(7주차)</v>
       </c>
       <c r="B6" t="str">
-        <v>24312002</v>
+        <v>24312005</v>
       </c>
       <c r="C6" t="str">
-        <v>강지구</v>
+        <v>김수빈</v>
       </c>
       <c r="D6" t="str">
-        <v>8번</v>
+        <v>-</v>
       </c>
       <c r="E6" t="str">
-        <v>26. 05. 07. 오후 07:37</v>
+        <v>26. 04. 16. 오후 07:00</v>
+      </c>
+      <c r="F6" t="str">
+        <v>2026-04-16T19:00:00</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>3회차(10주차)</v>
+        <v>2회차(7주차)</v>
       </c>
       <c r="B7" t="str">
-        <v>24312004</v>
+        <v>24312006</v>
       </c>
       <c r="C7" t="str">
-        <v>김석주</v>
+        <v>김유정</v>
       </c>
       <c r="D7" t="str">
-        <v>6번</v>
+        <v>-</v>
       </c>
       <c r="E7" t="str">
-        <v>26. 05. 07. 오후 07:37</v>
+        <v>26. 04. 16. 오후 07:00</v>
+      </c>
+      <c r="F7" t="str">
+        <v>2026-04-16T19:00:00</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>3회차(10주차)</v>
+        <v>2회차(7주차)</v>
       </c>
       <c r="B8" t="str">
-        <v>24312010</v>
+        <v>24312009</v>
       </c>
       <c r="C8" t="str">
-        <v>박지민</v>
+        <v>남진서</v>
       </c>
       <c r="D8" t="str">
-        <v>7번</v>
+        <v>-</v>
       </c>
       <c r="E8" t="str">
-        <v>26. 05. 07. 오후 07:37</v>
+        <v>26. 04. 16. 오후 07:00</v>
+      </c>
+      <c r="F8" t="str">
+        <v>2026-04-16T19:00:00</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>3회차(10주차)</v>
+        <v>2회차(7주차)</v>
       </c>
       <c r="B9" t="str">
-        <v>24312014</v>
+        <v>24312010</v>
       </c>
       <c r="C9" t="str">
-        <v>오준영</v>
+        <v>박지민</v>
       </c>
       <c r="D9" t="str">
-        <v>9번</v>
+        <v>-</v>
       </c>
       <c r="E9" t="str">
-        <v>26. 05. 07. 오후 07:37</v>
+        <v>26. 04. 16. 오후 07:00</v>
+      </c>
+      <c r="F9" t="str">
+        <v>2026-04-16T19:00:00</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>3회차(10주차)</v>
+        <v>2회차(7주차)</v>
       </c>
       <c r="B10" t="str">
-        <v>24312021</v>
+        <v>24312022</v>
       </c>
       <c r="C10" t="str">
-        <v>남궁민</v>
+        <v>변여아</v>
       </c>
       <c r="D10" t="str">
-        <v>2번</v>
+        <v>-</v>
       </c>
       <c r="E10" t="str">
-        <v>26. 05. 07. 오후 07:37</v>
+        <v>26. 04. 16. 오후 07:00</v>
+      </c>
+      <c r="F10" t="str">
+        <v>2026-04-16T19:00:00</v>
       </c>
     </row>
     <row r="11">
@@ -620,16 +662,19 @@
         <v>3회차(10주차)</v>
       </c>
       <c r="B11" t="str">
-        <v>24312023</v>
+        <v>24312002</v>
       </c>
       <c r="C11" t="str">
-        <v>송대원</v>
+        <v>강지구</v>
       </c>
       <c r="D11" t="str">
-        <v>1번</v>
+        <v>8번</v>
       </c>
       <c r="E11" t="str">
-        <v>26. 05. 07. 오후 07:37</v>
+        <v>26. 05. 07. 오후 07:00</v>
+      </c>
+      <c r="F11" t="str">
+        <v>2026-05-07T19:00:00</v>
       </c>
     </row>
     <row r="12">
@@ -637,28 +682,131 @@
         <v>3회차(10주차)</v>
       </c>
       <c r="B12" t="str">
+        <v>24312004</v>
+      </c>
+      <c r="C12" t="str">
+        <v>김석주</v>
+      </c>
+      <c r="D12" t="str">
+        <v>6번</v>
+      </c>
+      <c r="E12" t="str">
+        <v>26. 05. 07. 오후 07:00</v>
+      </c>
+      <c r="F12" t="str">
+        <v>2026-05-07T19:00:00</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>3회차(10주차)</v>
+      </c>
+      <c r="B13" t="str">
+        <v>24312010</v>
+      </c>
+      <c r="C13" t="str">
+        <v>박지민</v>
+      </c>
+      <c r="D13" t="str">
+        <v>7번</v>
+      </c>
+      <c r="E13" t="str">
+        <v>26. 05. 07. 오후 07:00</v>
+      </c>
+      <c r="F13" t="str">
+        <v>2026-05-07T19:00:00</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>3회차(10주차)</v>
+      </c>
+      <c r="B14" t="str">
+        <v>24312014</v>
+      </c>
+      <c r="C14" t="str">
+        <v>오준영</v>
+      </c>
+      <c r="D14" t="str">
+        <v>9번</v>
+      </c>
+      <c r="E14" t="str">
+        <v>26. 05. 07. 오후 07:00</v>
+      </c>
+      <c r="F14" t="str">
+        <v>2026-05-07T19:00:00</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>3회차(10주차)</v>
+      </c>
+      <c r="B15" t="str">
+        <v>24312021</v>
+      </c>
+      <c r="C15" t="str">
+        <v>남궁민</v>
+      </c>
+      <c r="D15" t="str">
+        <v>2번</v>
+      </c>
+      <c r="E15" t="str">
+        <v>26. 05. 07. 오후 07:00</v>
+      </c>
+      <c r="F15" t="str">
+        <v>2026-05-07T19:00:00</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>3회차(10주차)</v>
+      </c>
+      <c r="B16" t="str">
+        <v>24312023</v>
+      </c>
+      <c r="C16" t="str">
+        <v>송대원</v>
+      </c>
+      <c r="D16" t="str">
+        <v>1번</v>
+      </c>
+      <c r="E16" t="str">
+        <v>26. 05. 07. 오후 07:00</v>
+      </c>
+      <c r="F16" t="str">
+        <v>2026-05-07T19:00:00</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>3회차(10주차)</v>
+      </c>
+      <c r="B17" t="str">
         <v>24312030</v>
       </c>
-      <c r="C12" t="str">
+      <c r="C17" t="str">
         <v>조병현</v>
       </c>
-      <c r="D12" t="str">
+      <c r="D17" t="str">
         <v>4번</v>
       </c>
-      <c r="E12" t="str">
-        <v>26. 05. 07. 오후 07:37</v>
+      <c r="E17" t="str">
+        <v>26. 05. 07. 오후 07:00</v>
+      </c>
+      <c r="F17" t="str">
+        <v>2026-05-07T19:00:00</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F17"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:E12"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -673,69 +821,84 @@
       <c r="D1" t="str">
         <v>마지막 당첨일</v>
       </c>
+      <c r="E1" t="str">
+        <v>_마지막당첨일</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>24312005</v>
+        <v>24312010</v>
       </c>
       <c r="B2" t="str">
-        <v>김수빈</v>
+        <v>박지민</v>
       </c>
       <c r="C2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D2" t="str">
-        <v>2026. 4. 16.</v>
+        <v>2026. 5. 7.</v>
+      </c>
+      <c r="E2" t="str">
+        <v>2026-05-07T19:00:00</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>24312002</v>
+        <v>24312004</v>
       </c>
       <c r="B3" t="str">
-        <v>강지구</v>
+        <v>김석주</v>
       </c>
       <c r="C3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D3" t="str">
         <v>2026. 5. 7.</v>
       </c>
+      <c r="E3" t="str">
+        <v>2026-05-07T19:00:00</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>24312004</v>
+        <v>24312005</v>
       </c>
       <c r="B4" t="str">
-        <v>김석주</v>
+        <v>김수빈</v>
       </c>
       <c r="C4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D4" t="str">
-        <v>2026. 5. 7.</v>
+        <v>2026. 4. 16.</v>
+      </c>
+      <c r="E4" t="str">
+        <v>2026-04-16T19:00:00</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>24312006</v>
+        <v>24312009</v>
       </c>
       <c r="B5" t="str">
-        <v>김유정</v>
+        <v>남진서</v>
       </c>
       <c r="C5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D5" t="str">
         <v>2026. 4. 16.</v>
       </c>
+      <c r="E5" t="str">
+        <v>2026-04-16T19:00:00</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>24312010</v>
+        <v>24312002</v>
       </c>
       <c r="B6" t="str">
-        <v>박지민</v>
+        <v>강지구</v>
       </c>
       <c r="C6">
         <v>1</v>
@@ -743,27 +906,33 @@
       <c r="D6" t="str">
         <v>2026. 5. 7.</v>
       </c>
+      <c r="E6" t="str">
+        <v>2026-05-07T19:00:00</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>24312014</v>
+        <v>24312006</v>
       </c>
       <c r="B7" t="str">
-        <v>오준영</v>
+        <v>김유정</v>
       </c>
       <c r="C7">
         <v>1</v>
       </c>
       <c r="D7" t="str">
-        <v>2026. 5. 7.</v>
+        <v>2026. 4. 16.</v>
+      </c>
+      <c r="E7" t="str">
+        <v>2026-04-16T19:00:00</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>24312021</v>
+        <v>24312014</v>
       </c>
       <c r="B8" t="str">
-        <v>남궁민</v>
+        <v>오준영</v>
       </c>
       <c r="C8">
         <v>1</v>
@@ -771,41 +940,50 @@
       <c r="D8" t="str">
         <v>2026. 5. 7.</v>
       </c>
+      <c r="E8" t="str">
+        <v>2026-05-07T19:00:00</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>24312022</v>
+        <v>24312021</v>
       </c>
       <c r="B9" t="str">
-        <v>변여아</v>
+        <v>남궁민</v>
       </c>
       <c r="C9">
         <v>1</v>
       </c>
       <c r="D9" t="str">
-        <v>2026. 4. 16.</v>
+        <v>2026. 5. 7.</v>
+      </c>
+      <c r="E9" t="str">
+        <v>2026-05-07T19:00:00</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>24312023</v>
+        <v>24312022</v>
       </c>
       <c r="B10" t="str">
-        <v>송대원</v>
+        <v>변여아</v>
       </c>
       <c r="C10">
         <v>1</v>
       </c>
       <c r="D10" t="str">
-        <v>2026. 5. 7.</v>
+        <v>2026. 4. 16.</v>
+      </c>
+      <c r="E10" t="str">
+        <v>2026-04-16T19:00:00</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>24312030</v>
+        <v>24312023</v>
       </c>
       <c r="B11" t="str">
-        <v>조병현</v>
+        <v>송대원</v>
       </c>
       <c r="C11">
         <v>1</v>
@@ -813,10 +991,30 @@
       <c r="D11" t="str">
         <v>2026. 5. 7.</v>
       </c>
+      <c r="E11" t="str">
+        <v>2026-05-07T19:00:00</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>24312030</v>
+      </c>
+      <c r="B12" t="str">
+        <v>조병현</v>
+      </c>
+      <c r="C12">
+        <v>1</v>
+      </c>
+      <c r="D12" t="str">
+        <v>2026. 5. 7.</v>
+      </c>
+      <c r="E12" t="str">
+        <v>2026-05-07T19:00:00</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E12"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -868,7 +1066,7 @@
         <v>8번</v>
       </c>
       <c r="G2" t="str">
-        <v>26. 05. 07. 오후 07:21</v>
+        <v>26. 05. 11. 오전 10:05</v>
       </c>
     </row>
     <row r="3">
@@ -891,7 +1089,7 @@
         <v>6번</v>
       </c>
       <c r="G3" t="str">
-        <v>26. 05. 07. 오후 07:21</v>
+        <v>26. 05. 11. 오전 10:05</v>
       </c>
     </row>
     <row r="4">
@@ -914,7 +1112,7 @@
         <v>미배정</v>
       </c>
       <c r="G4" t="str">
-        <v>26. 05. 07. 오후 07:21</v>
+        <v>26. 05. 11. 오전 10:05</v>
       </c>
     </row>
     <row r="5">
@@ -937,7 +1135,7 @@
         <v>7번</v>
       </c>
       <c r="G5" t="str">
-        <v>26. 05. 07. 오후 07:20</v>
+        <v>26. 05. 11. 오전 10:05</v>
       </c>
     </row>
     <row r="6">
@@ -960,7 +1158,7 @@
         <v>9번</v>
       </c>
       <c r="G6" t="str">
-        <v>26. 05. 07. 오후 07:21</v>
+        <v>26. 05. 11. 오전 10:05</v>
       </c>
     </row>
     <row r="7">
@@ -983,7 +1181,7 @@
         <v>2번</v>
       </c>
       <c r="G7" t="str">
-        <v>26. 05. 07. 오후 07:22</v>
+        <v>26. 05. 11. 오전 10:05</v>
       </c>
     </row>
     <row r="8">
@@ -1006,7 +1204,7 @@
         <v>미배정</v>
       </c>
       <c r="G8" t="str">
-        <v>26. 05. 07. 오후 07:21</v>
+        <v>26. 05. 11. 오전 10:05</v>
       </c>
     </row>
     <row r="9">
@@ -1029,7 +1227,7 @@
         <v>1번</v>
       </c>
       <c r="G9" t="str">
-        <v>26. 05. 07. 오후 07:32</v>
+        <v>26. 05. 11. 오전 10:05</v>
       </c>
     </row>
     <row r="10">
@@ -1052,7 +1250,7 @@
         <v>4번</v>
       </c>
       <c r="G10" t="str">
-        <v>26. 05. 07. 오후 07:22</v>
+        <v>26. 05. 11. 오전 10:05</v>
       </c>
     </row>
   </sheetData>

</xml_diff>